<commit_message>
Remove Jobgether aggregator results from Rosalind's data and regenerate deliverables
Jobgether was explicitly excluded in ONE_CLICK config but 4 entries slipped through.
Removed from master database (18→14 jobs) and weekly CSVs. Regenerated xlsx and
analysis PDF with clean data and updated search optimization notes.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/For_Others/Rosalind_Gahamire/Week_of_2026-02-22/deliverables/Rosalind_Gahamire_Master_List_2026-02-22.xlsx
+++ b/results/For_Others/Rosalind_Gahamire/Week_of_2026-02-22/deliverables/Rosalind_Gahamire_Master_List_2026-02-22.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$5:$N$19</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,25 +28,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001F3864"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <color rgb="002F5496"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Helvetica"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
       <sz val="10"/>
     </font>
     <font>
@@ -53,23 +61,17 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00006100"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-        <bgColor rgb="001F3864"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -87,12 +89,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
         <bgColor rgb="00D6E4F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -133,37 +129,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -530,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -540,7 +545,7 @@
     <col width="35" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
@@ -556,22 +561,22 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Week of February 22, 2026  |  Prepared by Joey Clark</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Total Opportunities: 18 | Average Score: 78.7 | High Scores (80+): 8</t>
+          <t>14 jobs  |  Score range: 72-87  |  Avg: 80  |  14 NEW, 0 REPEAT</t>
         </is>
       </c>
     </row>
     <row r="4" ht="8" customHeight="1"/>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5" ht="25" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Status</t>
@@ -584,7 +589,8 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Score_Rationale</t>
+          <t>Score
+Rationale</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -594,7 +600,8 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Job_Title</t>
+          <t>Job
+Title</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -609,22 +616,26 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Language_Requirement</t>
+          <t>Language
+Requirement</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Work_Arrangement</t>
+          <t>Work
+Arrangement</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Salary_USD</t>
+          <t>Salary
+USD</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Job_Summary</t>
+          <t>Job
+Summary</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -634,12 +645,14 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>URL_Status</t>
+          <t>URL
+Status</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>Found_On</t>
+          <t>Found
+On</t>
         </is>
       </c>
     </row>
@@ -657,35 +670,35 @@
           <t>Excellent D2C creative strategy fit with direct overlap on brand strategy, insight-led research, visual storytelling, and creative direction. Portugal listed as eligible location. Timezone constraint (must align 3-4 hours with Singapore GMT+8) reduces location score slightly.</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Maneuver Marketing</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Creative Strategist</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>D2C Health &amp; Wellness</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Remote (Portugal eligible)</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <v/>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v/>
       </c>
       <c r="K6" s="7" t="inlineStr">
@@ -693,24 +706,24 @@
           <t>Drive high-converting, performance-driven creative assets for a $100M+ DTC supplements brand. Conduct in-depth visual research, develop creative testing strategies, manage ideation and execution of digital advertising assets across Meta platforms, and research competitor ad strategies. 5+ years in creative DTC advertising required.</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/maneuver-marketing/d5f90b21-1fcd-4503-8af9-899db0e1cf06</t>
         </is>
       </c>
-      <c r="M6" s="7" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
@@ -718,62 +731,62 @@
       <c r="B7" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Location: 30/30 (Remote-Global); Skills: 25/25 (Brand strategy, creative direction, insight-led research, messaging frameworks, stakeholder comms, design literacy); Industry: 20/20 (Creative agency); Salary: 12/15 (N/A); Seniority: 10/10 (Manager/Lead level)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Jobandtalent</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Director Brand Marketing</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Creative Agency</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>€120,000-€140,000 (approx)</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>Reports to SVP Brand and Communication. Drive awareness and recognition across 9+ markets in Europe, LATAM and US. Build distinct brand while creating strong brand experiences through sponsorships and TV activations. Remote-first company with team camps across Europe. Annual learning budget €1,000.</t>
         </is>
       </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="L7" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/jobandtalent/af7df888-3a4a-49ef-99d4-653c2ad369e8</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="M7" s="11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>jobs.lever.co</t>
         </is>
@@ -793,35 +806,35 @@
           <t>Strong brand strategy alignment as a player-coach Head of Marketing role in Lisbon. Covers brand and product marketing, creative studio, social media, influencer marketing, and PR. Consumer tech brand with 25M+ MAU. Head-level may be a stretch for 8 years experience but player-coach framing suggests hands-on work.</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Goodnotes</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Head of Marketing</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Consumer Tech / Productivity</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Lisbon, Portugal</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="8" t="n">
         <v/>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="8" t="n">
         <v/>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -829,24 +842,24 @@
           <t>Lead the Marketing function as a strategic leader and hands-on executor across Brand and Product Marketing, including creative studio, local marketing, social media &amp; influencer marketing, and PR. Drive creative campaigns and collaborate cross-functionally to elevate Goodnotes' global presence. Reports directly to leadership.</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="L8" s="8" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/goodnotes/jobs/5588098004</t>
         </is>
       </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
@@ -854,58 +867,58 @@
       <c r="B9" s="6" t="n">
         <v>84</v>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Lisbon-based fintech with strong overlap on brand positioning, messaging frameworks, and value propositions — core PMM skills that align directly with Rosalind's brand strategy experience. First PMM hire gives ownership and strategic influence. Fintech sector is outside target D2C/agency but has strong brand focus.</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>GetGround</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>Senior Product Marketing Manager - Fintech</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Fintech / Proptech</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Lisbon, Portugal</t>
         </is>
       </c>
-      <c r="H9" s="9" t="n">
+      <c r="H9" s="11" t="n">
         <v/>
       </c>
-      <c r="I9" s="9" t="inlineStr">
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="J9" s="9" t="n">
+      <c r="J9" s="11" t="n">
         <v/>
       </c>
-      <c r="K9" s="9" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>As the first PMM for GetGround Lisbon, own the product proposition and set product marketing best practices across the full product lifecycle. Define messaging and GTM strategy, launch features, and drive sustained adoption. Work closely with VP Product and team of PMs and Designers. Post-Series A from QED and Mosaic.</t>
         </is>
       </c>
-      <c r="L9" s="9" t="inlineStr">
+      <c r="L9" s="11" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/getground/jobs/4139448004</t>
         </is>
       </c>
-      <c r="M9" s="9" t="inlineStr">
+      <c r="M9" s="11" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="N9" s="9" t="inlineStr">
+      <c r="N9" s="11" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
@@ -925,37 +938,37 @@
           <t>Strong D2C creative strategy fit with CET timezone alignment (ideal for Lisbon). Owns creative pipeline from research to ad ideation and delivery for a Swiss D2C consumer brand. Skills overlap on creative strategy, competitive research, and team briefing. Salary range of $2-3K/month is significantly below market.</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Talo</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Creative Strategist</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>D2C Consumer Goods (Cleaning)</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Remote (European Economic Area)</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>German (huge plus but not required)</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>$24,000-$36,000/yr</t>
         </is>
@@ -965,24 +978,24 @@
           <t>Own the full creative pipeline for a fast-growing Swiss D2C cleaning brand — from competitor research to ad ideation, team briefing, and final delivery. Plan, brief, and produce high-performing Meta ad creatives. Lead a small creative team (copywriter, media buyer). CET timezone, 40hrs/week, plus 1% profit share.</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="L10" s="8" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/creative-strategist-at-talo-ai-4272176134</t>
         </is>
       </c>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Unverified</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
@@ -990,58 +1003,58 @@
       <c r="B11" s="6" t="n">
         <v>82</v>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Lisbon office option with integrated campaign strategy work across brand awareness and demand gen. Cross-functional collaboration with Design Studio, Product Marketing, and Creative teams overlaps with Rosalind's multi-stakeholder experience. B2B SaaS spend management sector rather than D2C, but involves brand-building.</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Pleo</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Integrated Campaigns Manager</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>B2B SaaS / Fintech</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Europe (London, Lisbon, Madrid, Copenhagen, Stockholm)</t>
         </is>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H11" s="11" t="n">
         <v/>
       </c>
-      <c r="I11" s="9" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="J11" s="9" t="n">
+      <c r="J11" s="11" t="n">
         <v/>
       </c>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>Lead creation of strategic, integrated marketing programs supporting Pleo's growth. Develop campaigns across email, social, website, video, events, and full-funnel collateral. Collaborate with Design Studio, Product Marketing, Performance, SEO, and Field Marketing teams. Reports to Head of Growth Marketing &amp; Demand Gen. 500+ team across 54 nations.</t>
         </is>
       </c>
-      <c r="L11" s="9" t="inlineStr">
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/pleo/jobs/4834700003</t>
         </is>
       </c>
-      <c r="M11" s="9" t="inlineStr">
+      <c r="M11" s="11" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
@@ -1061,37 +1074,37 @@
           <t>Location: 30/30 (Remote-Global); Skills: 25/25 (Brand strategy, creative direction, design literacy, workshop facilitation, stakeholder comms); Industry: 20/20 (Creative agency); Salary: 12/15 (N/A); Seniority: 10/10 (Manager/Lead level)</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>How&amp;How</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Brand Strategist</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Creative Agency</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>London/Lisbon</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Hybrid (London/Lisbon offices)</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>€55,000-€70,000 (est.)</t>
         </is>
@@ -1101,24 +1114,24 @@
           <t>Translate data and insights into actionable recommendations for creative team and clients. Work at intersection of strategy and creative execution. Talent-driven, creative culture. 11 full-time team. Works with tech and sustainability-focused brands.</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>https://www.ifyoucouldjobs.com/jobs/5726307320</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>ifyoucouldjobs.com</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
@@ -1126,62 +1139,62 @@
       <c r="B13" s="6" t="n">
         <v>80</v>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Location: 25/30 (Remote-Europe); Skills: 23/25 (Brand strategy, creative direction, campaign execution, messaging, stakeholder comms - limited design literacy); Industry: 20/20 (D2C brands); Salary: 15/15 (€1,500-€3,000/mo competitive); Seniority: 10/10 (Manager level)</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Foxelli Group</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>Brand Manager - DTC E-commerce</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>D2C Brands</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>Remote-Europe (EET timezone)</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr">
+      <c r="I13" s="11" t="inlineStr">
         <is>
           <t>Remote-Europe</t>
         </is>
       </c>
-      <c r="J13" s="9" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>€18,000-€36,000 (annually after-tax equivalent)</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>Own full-stack marketing role from ideation to sales execution. Bridge between marketing, design, development. Turn customer insights into landing pages, funnels, campaigns. Build brands generating €20M+ annually. Requires 5+ hours EET overlap.</t>
         </is>
       </c>
-      <c r="L13" s="9" t="inlineStr">
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>https://foxelligroup.recruitee.com/o/e-commerce-brand-manager-2</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr">
+      <c r="M13" s="11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N13" s="9" t="inlineStr">
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>recruitee.com</t>
         </is>
@@ -1193,7 +1206,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="12" t="n">
         <v>79</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -1201,37 +1214,37 @@
           <t>Location: 25/30 (Remote-Europe); Skills: 22/25 (Creative direction, campaign development, performance analysis, brand strategy); Industry: 20/20 (D2C brands); Salary: 12/15 (N/A listed); Seniority: 8/10 (Lead level)</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Foxelli Group</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Marketing Manager - DTC E-commerce</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>D2C Brands</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>Remote-Europe (EET timezone)</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>Remote-Europe</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>€18,000-€36,000 (annually after-tax equivalent)</t>
         </is>
@@ -1241,87 +1254,87 @@
           <t>Full-stack marketing ownership. Think big, move fast. Bridge between marketing, design, development. Turn insights into landing pages, funnels, campaigns. Work in EET timezone. Foxelli builds D2C brands with €20M+ annual revenue.</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>https://nploy.net/jobs/marketing-and-communications-pr/remote-multiple-locations/marketing-manager-or-dtc-e-commerce-or-100percent-remote-eu1770889177/217527-X</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>nPloy</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="12" t="n">
         <v>78</v>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Location: 30/30 (Remote-Global); Skills: 20/25 (Performance creative analysis, campaign development, brief execution - limited strategy depth); Industry: 15/20 (Consumer tech/performance focus); Salary: 15/15 ($67,900-$102,100 range); Seniority: 10/10 (Senior/Manager level)</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Monks</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>Senior Creative Strategist, Performance Creative</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Performance Marketing Agency</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>Remote (US/Global)</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="I15" s="9" t="inlineStr">
+      <c r="I15" s="11" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="J15" s="9" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
         <is>
           <t>$67,900-$102,100</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>Report to Director of Creative Strategy. Lead creative conversation with clients. Improve performance through testing and cultural insights. Weekly/monthly reporting, concept briefing, creative testing expertise. 3-5+ years client-facing strategic role required. Facebook, Instagram, TikTok, LinkedIn mandatory.</t>
         </is>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="L15" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/monks/jobs/5697740004</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M15" s="11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="N15" s="11" t="inlineStr">
         <is>
           <t>greenhouse.io</t>
         </is>
@@ -1333,7 +1346,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="12" t="n">
         <v>77</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -1341,35 +1354,35 @@
           <t>Lisbon-based consumer tech company with 100M+ downloads and offices in Lisbon and San Francisco. Digital marketing execution focus rather than brand strategy, with limited overlap on Rosalind's core strategic skills. Good location and consumer industry fit but more hands-on digital marketing than strategic.</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Air Apps</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Digital Marketing Manager</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Consumer Tech / Mobile Apps</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Lisbon, Portugal</t>
         </is>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H16" s="8" t="n">
         <v/>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>In-Office</t>
         </is>
       </c>
-      <c r="J16" s="7" t="n">
+      <c r="J16" s="8" t="n">
         <v/>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -1377,87 +1390,87 @@
           <t>Plan, execute, and optimize online marketing campaigns across multiple channels for an AI-powered personal resource planner. Born in Lisbon in 2018 with 100M+ downloads worldwide, self-funded with offices in Lisbon and San Francisco. Responsible for campaign strategy and performance optimization.</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/airapps/6e89f68d-bad6-4755-950f-10b537c191d5</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="N16" s="7" t="inlineStr">
+      <c r="N16" s="8" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="12" t="n">
         <v>76</v>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Location: 30/30 (Remote-Global); Skills: 20/25 (Creative strategy, brand development, design literacy, workshop facilitation - limited research); Industry: 15/20 (D2C consumer brands); Salary: 12/15 (N/A); Seniority: 10/10 (Manager/Senior level)</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Grüns</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Creative Strategist</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>D2C Brands</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr">
+      <c r="I17" s="11" t="inlineStr">
         <is>
           <t>Fully Remote</t>
         </is>
       </c>
-      <c r="J17" s="9" t="inlineStr">
+      <c r="J17" s="11" t="inlineStr">
         <is>
           <t>€55,000-€75,000 (est.)</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>Drive creative direction and strategy for high-performing ad creative across Meta, YouTube, TikTok. Fully remote, high-trust environment with bi-annual in-person off-sites. Work with designers, video editors, external creators. Optimize conversion-focused performance. Nutrition/CPG sector.</t>
         </is>
       </c>
-      <c r="L17" s="9" t="inlineStr">
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gruns/jobs/4976473008</t>
         </is>
       </c>
-      <c r="M17" s="9" t="inlineStr">
+      <c r="M17" s="11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="N17" s="11" t="inlineStr">
         <is>
           <t>greenhouse.io</t>
         </is>
@@ -1469,414 +1482,143 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n">
-        <v>75</v>
+      <c r="B18" s="12" t="n">
+        <v>74</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Location: 25/30 (Remote-Europe); Skills: 22/25 (Brand strategy, creative direction, communications, stakeholder management, limited design literacy); Industry: 15/20 (B2B with brand focus); Salary: 12/15 (N/A); Seniority: 8/10 (Director/Senior level)</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Jobgether (Partner Company)</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Head of Brand Strategy</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Various Sectors</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Remote-Europe/Global</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
+          <t>Excellent Lisbon location with hybrid flexibility across Portugal. First marketing hire in Lisbon for a European VC. Growth marketing across paid and organic channels for diverse portfolio companies. Limited brand strategy overlap — more execution-focused performance marketing than strategic brand work.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Project A</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Senior Growth Marketing Manager</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Venture Capital / Portfolio Services</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Lisbon, Portugal</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v/>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>First marketing hire in Lisbon for a leading European VC. Execute marketing strategies across organic and paid channels for diverse portfolio companies. Join a team of data-driven experts covering programmatic paid media, demand generation, marketing automation, and MarTech. EU work eligibility required.</t>
+        </is>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/projectaservicesgmbhcokg/jobs/7725674002</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Remote Portugal role with product marketing focus bridging product and customer needs. Non-profit fundraising tech sector is outside target D2C/agency industries. Some overlap on positioning, messaging, and cross-functional collaboration but limited brand strategy alignment.</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Fundraise Up</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Product Marketing Manager</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Non-Profit Tech / SaaS</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Portugal (Remote)</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>Remote-Global</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>€90,000-€120,000 (est.)</t>
-        </is>
-      </c>
-      <c r="K18" s="7" t="inlineStr">
-        <is>
-          <t>Shape and unify corporate brand narrative across diverse product portfolio. Elevate brand as industry leader. Strategic and creative positioning. Lead brand communication and messaging across markets.</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/jobgether/92363484-d8e9-4ae1-9bdc-605a9c100dac</t>
-        </is>
-      </c>
-      <c r="M18" s="7" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N18" s="7" t="inlineStr">
-        <is>
-          <t>jobs.lever.co</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="n">
-        <v>74</v>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Excellent Lisbon location with hybrid flexibility across Portugal. First marketing hire in Lisbon for a European VC. Growth marketing across paid and organic channels for diverse portfolio companies. Limited brand strategy overlap — more execution-focused performance marketing than strategic brand work.</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>Project A</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>Senior Growth Marketing Manager</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>Venture Capital / Portfolio Services</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Lisbon, Portugal</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="n">
+      <c r="J19" s="11" t="n">
         <v/>
       </c>
-      <c r="I19" s="9" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J19" s="9" t="n">
-        <v/>
-      </c>
-      <c r="K19" s="9" t="inlineStr">
-        <is>
-          <t>First marketing hire in Lisbon for a leading European VC. Execute marketing strategies across organic and paid channels for diverse portfolio companies. Join a team of data-driven experts covering programmatic paid media, demand generation, marketing automation, and MarTech. EU work eligibility required.</t>
-        </is>
-      </c>
-      <c r="L19" s="9" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/projectaservicesgmbhcokg/jobs/7725674002</t>
-        </is>
-      </c>
-      <c r="M19" s="9" t="inlineStr">
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>Bridge the gap between product offerings and customer needs for the leading non-profit fundraising platform. Collaborate with marketing, engineering, sales, and customer success teams. UNICEF, Alzheimer's Association, and other major non-profits use the platform. Remote role based in Portugal.</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/fundraiseup/jobs/4501944005</t>
+        </is>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="N19" s="11" t="inlineStr">
         <is>
           <t>Greenhouse</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>74</v>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Location: 30/30 (Remote-Global); Skills: 18/25 (Messaging frameworks, campaign execution, brand comms - limited strategic depth); Industry: 15/20 (Consumer tech); Salary: 12/15 (N/A); Seniority: 10/10 (Manager level)</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Jobgether (Partner Company)</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Head of Communications &amp; Brand Strategy</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Various Sectors</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Remote-Europe/Global</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>Remote-Global</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>€85,000-€110,000 (est.)</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>Communications leadership role focused on brand strategy execution. Shape brand narrative. Create strong brand experiences. Remote-first structure with European operations.</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>https://jobgether.com/offer/6976d1d073a8e8b5e77b5dc8-head-of-communications-brand-strategy-europe-or-u.s.---remote</t>
-        </is>
-      </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N20" s="7" t="inlineStr">
-        <is>
-          <t>jobgether.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="n">
-        <v>73</v>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Location: 25/30 (Remote-Europe); Skills: 20/25 (Brand strategy, creative direction, campaign development, stakeholder comms - limited research); Industry: 20/20 (Creative agency); Salary: 12/15 (N/A); Seniority: 8/10 (Senior/Lead level)</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Jobgether (Partner Company)</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>Remote Brand Creative Strategist</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Creative Agency/Multiple</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>Remote-Europe</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="I21" s="9" t="inlineStr">
-        <is>
-          <t>Remote-Europe</t>
-        </is>
-      </c>
-      <c r="J21" s="9" t="inlineStr">
-        <is>
-          <t>€70,000-€95,000 (est.)</t>
-        </is>
-      </c>
-      <c r="K21" s="9" t="inlineStr">
-        <is>
-          <t>Marketing Creative Strategist in dynamic team designing innovative marketing strategies. 5+ years in creative design. Develop brand concepts and campaign strategies. Strategic positioning and creative execution.</t>
-        </is>
-      </c>
-      <c r="L21" s="9" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/jobgether/e80249e8-89c2-4448-a441-f1549604183c</t>
-        </is>
-      </c>
-      <c r="M21" s="9" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N21" s="9" t="inlineStr">
-        <is>
-          <t>jobs.lever.co</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>72</v>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Remote Portugal role with product marketing focus bridging product and customer needs. Non-profit fundraising tech sector is outside target D2C/agency industries. Some overlap on positioning, messaging, and cross-functional collaboration but limited brand strategy alignment.</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Fundraise Up</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>Product Marketing Manager</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Non-Profit Tech / SaaS</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Portugal (Remote)</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>Remote-Global</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v/>
-      </c>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>Bridge the gap between product offerings and customer needs for the leading non-profit fundraising platform. Collaborate with marketing, engineering, sales, and customer success teams. UNICEF, Alzheimer's Association, and other major non-profits use the platform. Remote role based in Portugal.</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/fundraiseup/jobs/4501944005</t>
-        </is>
-      </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="N22" s="7" t="inlineStr">
-        <is>
-          <t>Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n">
-        <v>71</v>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Location: 25/30 (Remote-Europe); Skills: 18/25 (Brand marketing, campaign execution, creative direction - limited strategic research); Industry: 15/20 (Consumer tech/B2B); Salary: 12/15 (N/A); Seniority: 10/10 (Manager level)</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Jobgether (Partner Company)</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Remote Brand Marketing Manager</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Various Sectors</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Remote-Europe</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Remote-Europe</t>
-        </is>
-      </c>
-      <c r="J23" s="9" t="inlineStr">
-        <is>
-          <t>€75,000-€95,000 (est.)</t>
-        </is>
-      </c>
-      <c r="K23" s="9" t="inlineStr">
-        <is>
-          <t>Brand marketing leadership in European market. Execute marketing strategies and brand campaigns. Remote team-first environment. Build brand recognition and market positioning.</t>
-        </is>
-      </c>
-      <c r="L23" s="9" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/jobgether/8f4c90f5-a2fe-490b-830a-bc8d6de13445</t>
-        </is>
-      </c>
-      <c r="M23" s="9" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N23" s="9" t="inlineStr">
-        <is>
-          <t>jobs.lever.co</t>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Score Key:  🟢 90+ Elite  |  🔵 80-89 Strong  |  🟡 70-79 Good  |  🔴 Below 70</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <autoFilter ref="A5:N19"/>
+  <mergeCells count="4">
+    <mergeCell ref="A21:N21"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>